<commit_message>
Update Stundenliste (Better and more enhanced version = weniger Valentins auf der Seite)
</commit_message>
<xml_diff>
--- a/Stundenliste_neu(1)(1)(1).xlsx
+++ b/Stundenliste_neu(1)(1)(1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VR2\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arthur\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77CB59CF-1063-4FB8-B52D-6451E03B4701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE690E5-7B73-42E2-8767-720FF2144877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{904973F5-B02B-4666-A03D-BB66738E721E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{904973F5-B02B-4666-A03D-BB66738E721E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="111">
   <si>
     <t>Tag</t>
   </si>
@@ -366,6 +366,9 @@
   </si>
   <si>
     <t>Hand Teleportation</t>
+  </si>
+  <si>
+    <t>Diplomarbeitstext Zusammenfassung</t>
   </si>
 </sst>
 </file>
@@ -465,7 +468,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -499,11 +502,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Prozent" xfId="1" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
@@ -720,7 +722,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="de-DE"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -982,7 +984,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.99232456140350367</c:v>
+                  <c:v>0.99780701754385415</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2049,9 +2051,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2089,7 +2091,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2195,7 +2197,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2384,7 +2386,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{730198CE-52B5-4F02-9B4B-1774B163D30B}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:U119"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" customWidth="1"/>
@@ -2559,23 +2561,23 @@
       </c>
       <c r="M4" s="11">
         <f>SUM(J5,J8,J9,J11)</f>
-        <v>7.5416666666666661</v>
+        <v>7.5833333333333321</v>
       </c>
       <c r="N4" s="18">
         <f t="shared" ref="N4:N5" si="2">M4</f>
-        <v>7.5416666666666661</v>
+        <v>7.5833333333333321</v>
       </c>
       <c r="O4" s="18">
         <f t="shared" ref="O4:O5" si="3">N4/60</f>
-        <v>0.12569444444444444</v>
+        <v>0.12638888888888886</v>
       </c>
       <c r="P4" s="22">
         <f t="shared" si="1"/>
-        <v>6.9830246913580252E-2</v>
+        <v>7.0216049382716028E-2</v>
       </c>
       <c r="Q4" s="21">
         <f t="shared" ref="Q4:Q5" si="4">(P4*1421.05263157894)/100</f>
-        <v>0.99232456140350367</v>
+        <v>0.99780701754385415</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
@@ -2607,7 +2609,7 @@
       </c>
       <c r="J5" s="10">
         <f>SUMIF(Stundenliste[Wer],I5,Stundenliste[Stunden])</f>
-        <v>2.875</v>
+        <v>2.9166666666666665</v>
       </c>
       <c r="L5" t="s">
         <v>9</v>
@@ -2709,7 +2711,7 @@
       </c>
       <c r="M7" s="15">
         <f>SUM(F2:F119)</f>
-        <v>12.541666666666671</v>
+        <v>12.583333333333337</v>
       </c>
       <c r="N7">
         <v>180</v>
@@ -2748,7 +2750,7 @@
       </c>
       <c r="M8" s="16">
         <f>TEXT(M7,"[h]")+TEXT(M7,"mm")/60</f>
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
@@ -5102,14 +5104,14 @@
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A102" s="23" t="str">
+      <c r="A102" s="2" t="str">
         <f>IF(ISNUMBER(B102),LEFT(TEXT(B102,"TTTT"),2)&amp;".","")</f>
         <v>Fr.</v>
       </c>
       <c r="B102" s="3">
         <v>46101</v>
       </c>
-      <c r="C102" s="23" t="s">
+      <c r="C102" s="2" t="s">
         <v>106</v>
       </c>
       <c r="D102" s="4">
@@ -5127,14 +5129,14 @@
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A103" s="23" t="str">
+      <c r="A103" s="2" t="str">
         <f>IF(ISNUMBER(B103),LEFT(TEXT(B103,"TTTT"),2)&amp;".","")</f>
         <v>Do.</v>
       </c>
       <c r="B103" s="3">
         <v>46100</v>
       </c>
-      <c r="C103" s="23" t="s">
+      <c r="C103" s="2" t="s">
         <v>107</v>
       </c>
       <c r="D103" s="4">
@@ -5152,14 +5154,14 @@
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" s="23" t="str">
+      <c r="A104" s="2" t="str">
         <f>IF(ISNUMBER(B104),LEFT(TEXT(B104,"TTTT"),2)&amp;".","")</f>
         <v>Do.</v>
       </c>
       <c r="B104" s="3">
         <v>46086</v>
       </c>
-      <c r="C104" s="23" t="s">
+      <c r="C104" s="2" t="s">
         <v>109</v>
       </c>
       <c r="D104" s="4">
@@ -5177,169 +5179,155 @@
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" s="23"/>
-      <c r="B105" s="3"/>
-      <c r="C105" s="23"/>
-      <c r="D105" s="4"/>
-      <c r="E105" s="4"/>
-      <c r="F105" s="5"/>
+      <c r="A105" s="2" t="str">
+        <f>IF(ISNUMBER(B105),LEFT(TEXT(B105,"TTTT"),2)&amp;".","")</f>
+        <v>So.</v>
+      </c>
+      <c r="B105" s="3">
+        <v>46103</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D105" s="4">
+        <v>0.875</v>
+      </c>
+      <c r="E105" s="4">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F105" s="5">
+        <f>IF(E105&gt;D105,E105-D105,IF(ISNUMBER(Stundenliste[[#This Row],[Von]]),"24:00"-(D105-E105),""))</f>
+        <v>4.166666666666663E-2</v>
+      </c>
       <c r="G105" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A106" s="23"/>
+      <c r="A106" s="2"/>
       <c r="B106" s="3"/>
-      <c r="C106" s="23"/>
+      <c r="C106" s="2"/>
       <c r="D106" s="4"/>
       <c r="E106" s="4"/>
       <c r="F106" s="5"/>
-      <c r="G106" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G106" s="2"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A107" s="23"/>
+      <c r="A107" s="2"/>
       <c r="B107" s="3"/>
-      <c r="C107" s="23"/>
+      <c r="C107" s="2"/>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
       <c r="F107" s="5"/>
-      <c r="G107" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G107" s="2"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A108" s="23"/>
+      <c r="A108" s="2"/>
       <c r="B108" s="3"/>
-      <c r="C108" s="23"/>
+      <c r="C108" s="2"/>
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
       <c r="F108" s="5"/>
-      <c r="G108" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G108" s="2"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A109" s="23"/>
+      <c r="A109" s="2"/>
       <c r="B109" s="3"/>
-      <c r="C109" s="23"/>
+      <c r="C109" s="2"/>
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="5"/>
-      <c r="G109" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G109" s="2"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A110" s="23"/>
+      <c r="A110" s="2"/>
       <c r="B110" s="3"/>
-      <c r="C110" s="23"/>
+      <c r="C110" s="2"/>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
       <c r="F110" s="5"/>
-      <c r="G110" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G110" s="2"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A111" s="23"/>
+      <c r="A111" s="2"/>
       <c r="B111" s="3"/>
-      <c r="C111" s="23"/>
+      <c r="C111" s="2"/>
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
       <c r="F111" s="5"/>
-      <c r="G111" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G111" s="2"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" s="23"/>
+      <c r="A112" s="2"/>
       <c r="B112" s="3"/>
-      <c r="C112" s="23"/>
+      <c r="C112" s="2"/>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
       <c r="F112" s="5"/>
-      <c r="G112" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G112" s="2"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" s="23"/>
+      <c r="A113" s="2"/>
       <c r="B113" s="3"/>
-      <c r="C113" s="23"/>
+      <c r="C113" s="2"/>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="5"/>
-      <c r="G113" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G113" s="2"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A114" s="23"/>
+      <c r="A114" s="2"/>
       <c r="B114" s="3"/>
-      <c r="C114" s="23"/>
+      <c r="C114" s="2"/>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="5"/>
-      <c r="G114" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G114" s="2"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A115" s="23"/>
+      <c r="A115" s="2"/>
       <c r="B115" s="3"/>
-      <c r="C115" s="23"/>
+      <c r="C115" s="2"/>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
       <c r="F115" s="5"/>
-      <c r="G115" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G115" s="2"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A116" s="23"/>
+      <c r="A116" s="2"/>
       <c r="B116" s="3"/>
-      <c r="C116" s="23"/>
+      <c r="C116" s="2"/>
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
       <c r="F116" s="5"/>
-      <c r="G116" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G116" s="2"/>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A117" s="23"/>
+      <c r="A117" s="2"/>
       <c r="B117" s="3"/>
-      <c r="C117" s="23"/>
+      <c r="C117" s="2"/>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="5"/>
-      <c r="G117" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G117" s="2"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A118" s="23"/>
+      <c r="A118" s="2"/>
       <c r="B118" s="3"/>
-      <c r="C118" s="23"/>
+      <c r="C118" s="2"/>
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
       <c r="F118" s="5"/>
-      <c r="G118" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G118" s="2"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A119" s="23"/>
+      <c r="A119" s="2"/>
       <c r="B119" s="3"/>
-      <c r="C119" s="23"/>
+      <c r="C119" s="2"/>
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
       <c r="F119" s="5"/>
-      <c r="G119" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G119" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -5354,20 +5342,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ReferenceId xmlns="d9f85066-e658-4e34-914c-f198c2427564" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ReferenceId xmlns="d9f85066-e658-4e34-914c-f198c2427564" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5515,14 +5503,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A879EED-63D4-4BD6-ABDC-8DEB19CAAEDF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57E083A2-B59E-4178-BBDB-6F72551558F7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -5536,6 +5516,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="becce21f-4543-4ee3-84d8-746b4cf7c34b"/>
     <ds:schemaRef ds:uri="d9f85066-e658-4e34-914c-f198c2427564"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A879EED-63D4-4BD6-ABDC-8DEB19CAAEDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>